<commit_message>
migrated existing scan to django and made it also push to a websocket
</commit_message>
<xml_diff>
--- a/start_documents/planning.xlsx
+++ b/start_documents/planning.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mijn Drive\Stage WLW\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\debeer360\Desktop\school\WLW\start_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9019C7D-63B1-4CDF-B39E-86CC37D58765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A09BE50-93FF-4F05-9E14-B00571739B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F333C256-9A40-4403-A263-597E23E7B60C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>datum</t>
   </si>
@@ -105,6 +105,9 @@
   </si>
   <si>
     <t>Laatste meters maken/ thuiswerkperiode</t>
+  </si>
+  <si>
+    <t>Herkansing expert software development</t>
   </si>
 </sst>
 </file>
@@ -256,14 +259,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -274,11 +276,9 @@
     <xf numFmtId="14" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -623,7 +623,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -635,209 +635,209 @@
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="7">
         <v>46055</v>
       </c>
-      <c r="D2" s="3"/>
+      <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>46056</v>
       </c>
-      <c r="D3" s="3"/>
+      <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>46057</v>
       </c>
-      <c r="D4" s="3"/>
+      <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>46058</v>
       </c>
-      <c r="D5" s="3"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>46059</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>46060</v>
       </c>
-      <c r="D7" s="3"/>
+      <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <v>46061</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="8">
         <v>46062</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <v>46063</v>
       </c>
-      <c r="D10" s="3"/>
+      <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <v>46064</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="8">
         <v>46065</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="9">
+      <c r="B13" s="8">
         <v>46066</v>
       </c>
-      <c r="D13" s="3"/>
+      <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>46067</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="8">
         <v>46068</v>
       </c>
-      <c r="D15" s="3"/>
+      <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <v>46069</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="8">
         <v>46070</v>
       </c>
-      <c r="D17" s="3"/>
+      <c r="D17" s="1"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>46071</v>
       </c>
-      <c r="D18" s="3"/>
+      <c r="D18" s="1"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <v>46072</v>
       </c>
-      <c r="D19" s="3"/>
+      <c r="D19" s="1"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>46073</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="1"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="9">
+      <c r="A21" s="4"/>
+      <c r="B21" s="8">
         <v>46074</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="1"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="9">
+      <c r="B22" s="8">
         <v>46075</v>
       </c>
-      <c r="D22" s="3"/>
+      <c r="D22" s="1"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B23" s="6">
+      <c r="B23" s="5">
         <v>46076</v>
       </c>
-      <c r="D23" s="3"/>
+      <c r="D23" s="1"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="6">
         <v>46077</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="1"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="7">
+      <c r="B25" s="6">
         <v>46078</v>
       </c>
       <c r="D25" s="1"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="7">
+      <c r="B26" s="6">
         <v>46079</v>
       </c>
       <c r="D26" s="1"/>
@@ -846,7 +846,7 @@
       <c r="A27" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="7">
+      <c r="B27" s="6">
         <v>46080</v>
       </c>
       <c r="D27" s="1"/>
@@ -855,28 +855,28 @@
       <c r="A28" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="12">
+      <c r="B28" s="11">
         <v>46081</v>
       </c>
       <c r="D28" s="1"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
-      <c r="B29" s="13">
+      <c r="B29" s="12">
         <v>46082</v>
       </c>
       <c r="D29" s="1"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
-      <c r="B30" s="14">
+      <c r="B30" s="12">
         <v>46083</v>
       </c>
       <c r="D30" s="1"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
-      <c r="B31" s="14">
+      <c r="B31" s="12">
         <v>46084</v>
       </c>
       <c r="C31" t="s">
@@ -886,832 +886,835 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
-      <c r="B32" s="14">
+      <c r="B32" s="12">
         <v>46085</v>
       </c>
       <c r="D32" s="1"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
-      <c r="B33" s="14">
+      <c r="B33" s="12">
         <v>46086</v>
       </c>
       <c r="D33" s="1"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
-      <c r="B34" s="14">
+      <c r="B34" s="12">
         <v>46087</v>
       </c>
       <c r="D34" s="1"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
-      <c r="B35" s="14">
+      <c r="B35" s="12">
         <v>46088</v>
       </c>
       <c r="D35" s="1"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
-      <c r="B36" s="14">
+      <c r="B36" s="12">
         <v>46089</v>
       </c>
       <c r="D36" s="1"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
-      <c r="B37" s="14">
+      <c r="B37" s="12">
         <v>46090</v>
       </c>
       <c r="D37" s="1"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
-      <c r="B38" s="14">
+      <c r="B38" s="12">
         <v>46091</v>
       </c>
       <c r="D38" s="1"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
-      <c r="B39" s="14">
+      <c r="B39" s="12">
         <v>46092</v>
       </c>
       <c r="D39" s="1"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="14">
+      <c r="B40" s="12">
         <v>46093</v>
       </c>
       <c r="D40" s="1"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="14">
+      <c r="B41" s="12">
         <v>46094</v>
       </c>
       <c r="D41" s="1"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="14">
+      <c r="B42" s="12">
         <v>46095</v>
       </c>
       <c r="D42" s="1"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
-      <c r="B43" s="14">
+      <c r="B43" s="12">
         <v>46096</v>
       </c>
       <c r="D43" s="1"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
-      <c r="B44" s="14">
+      <c r="B44" s="12">
         <v>46097</v>
       </c>
       <c r="D44" s="1"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
-      <c r="B45" s="14">
+      <c r="B45" s="12">
         <v>46098</v>
       </c>
       <c r="D45" s="1"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
-      <c r="B46" s="14">
+      <c r="B46" s="12">
         <v>46099</v>
       </c>
       <c r="D46" s="1"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
-      <c r="B47" s="14">
+      <c r="B47" s="12">
         <v>46100</v>
       </c>
       <c r="D47" s="1"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
-      <c r="B48" s="14">
+      <c r="B48" s="12">
         <v>46101</v>
       </c>
       <c r="D48" s="1"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
-      <c r="B49" s="14">
+      <c r="B49" s="12">
         <v>46102</v>
       </c>
       <c r="D49" s="1"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
-      <c r="B50" s="14">
+      <c r="B50" s="12">
         <v>46103</v>
       </c>
       <c r="D50" s="1"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
-      <c r="B51" s="14">
+      <c r="B51" s="12">
         <v>46104</v>
+      </c>
+      <c r="C51" t="s">
+        <v>23</v>
       </c>
       <c r="D51" s="1"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
-      <c r="B52" s="14">
+      <c r="B52" s="12">
         <v>46105</v>
       </c>
       <c r="D52" s="1"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
-      <c r="B53" s="14">
+      <c r="B53" s="12">
         <v>46106</v>
       </c>
       <c r="D53" s="1"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
-      <c r="B54" s="14">
+      <c r="B54" s="12">
         <v>46107</v>
       </c>
       <c r="D54" s="1"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
-      <c r="B55" s="14">
+      <c r="B55" s="12">
         <v>46108</v>
       </c>
       <c r="D55" s="1"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
-      <c r="B56" s="14">
+      <c r="B56" s="12">
         <v>46109</v>
       </c>
       <c r="D56" s="1"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
-      <c r="B57" s="14">
+      <c r="B57" s="12">
         <v>46110</v>
       </c>
       <c r="D57" s="1"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
-      <c r="B58" s="14">
+      <c r="B58" s="12">
         <v>46111</v>
       </c>
       <c r="D58" s="1"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
-      <c r="B59" s="14">
+      <c r="B59" s="12">
         <v>46112</v>
       </c>
       <c r="D59" s="1"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
-      <c r="B60" s="14">
+      <c r="B60" s="12">
         <v>46113</v>
       </c>
       <c r="D60" s="1"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
-      <c r="B61" s="14">
+      <c r="B61" s="12">
         <v>46114</v>
       </c>
       <c r="D61" s="1"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
-      <c r="B62" s="14">
+      <c r="B62" s="12">
         <v>46115</v>
       </c>
       <c r="D62" s="1"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
-      <c r="B63" s="14">
+      <c r="B63" s="12">
         <v>46116</v>
       </c>
       <c r="D63" s="1"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
-      <c r="B64" s="14">
+      <c r="B64" s="12">
         <v>46117</v>
       </c>
       <c r="D64" s="1"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
-      <c r="B65" s="14">
+      <c r="B65" s="12">
         <v>46118</v>
       </c>
       <c r="D65" s="1"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
-      <c r="B66" s="14">
+      <c r="B66" s="12">
         <v>46119</v>
       </c>
       <c r="D66" s="1"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
-      <c r="B67" s="14">
+      <c r="B67" s="12">
         <v>46120</v>
       </c>
       <c r="D67" s="1"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
-      <c r="B68" s="14">
+      <c r="B68" s="12">
         <v>46121</v>
       </c>
       <c r="D68" s="1"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
-      <c r="B69" s="14">
+      <c r="B69" s="12">
         <v>46122</v>
       </c>
       <c r="D69" s="1"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
-      <c r="B70" s="14">
+      <c r="B70" s="12">
         <v>46123</v>
       </c>
       <c r="D70" s="1"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="1"/>
-      <c r="B71" s="14">
+      <c r="B71" s="12">
         <v>46124</v>
       </c>
       <c r="D71" s="1"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
-      <c r="B72" s="10">
+      <c r="B72" s="9">
         <v>46125</v>
       </c>
       <c r="D72" s="1"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
-      <c r="B73" s="10">
+      <c r="B73" s="9">
         <v>46126</v>
       </c>
       <c r="D73" s="1"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
-      <c r="B74" s="10">
+      <c r="B74" s="9">
         <v>46127</v>
       </c>
       <c r="D74" s="1"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
-      <c r="B75" s="10">
+      <c r="B75" s="9">
         <v>46128</v>
       </c>
       <c r="D75" s="1"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
-      <c r="B76" s="10">
+      <c r="B76" s="9">
         <v>46129</v>
       </c>
       <c r="D76" s="1"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="1"/>
-      <c r="B77" s="10">
+      <c r="B77" s="9">
         <v>46130</v>
       </c>
       <c r="D77" s="1"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
-      <c r="B78" s="10">
+      <c r="B78" s="9">
         <v>46131</v>
       </c>
       <c r="D78" s="1"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="1"/>
-      <c r="B79" s="10">
+      <c r="B79" s="9">
         <v>46132</v>
       </c>
       <c r="D79" s="1"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
-      <c r="B80" s="10">
+      <c r="B80" s="9">
         <v>46133</v>
       </c>
       <c r="D80" s="1"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
-      <c r="B81" s="10">
+      <c r="B81" s="9">
         <v>46134</v>
       </c>
       <c r="D81" s="1"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="1"/>
-      <c r="B82" s="10">
+      <c r="B82" s="9">
         <v>46135</v>
       </c>
       <c r="D82" s="1"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="1"/>
-      <c r="B83" s="10">
+      <c r="B83" s="9">
         <v>46136</v>
       </c>
       <c r="D83" s="1"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
-      <c r="B84" s="11">
+      <c r="B84" s="10">
         <v>46137</v>
       </c>
       <c r="D84" s="1"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
-      <c r="B85" s="11">
+      <c r="B85" s="10">
         <v>46138</v>
       </c>
       <c r="D85" s="1"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
-      <c r="B86" s="11">
+      <c r="B86" s="10">
         <v>46139</v>
       </c>
       <c r="D86" s="1"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
-      <c r="B87" s="11">
+      <c r="B87" s="10">
         <v>46140</v>
       </c>
       <c r="D87" s="1"/>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
-      <c r="B88" s="11">
+      <c r="B88" s="10">
         <v>46141</v>
       </c>
       <c r="D88" s="1"/>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
-      <c r="B89" s="11">
+      <c r="B89" s="10">
         <v>46142</v>
       </c>
       <c r="D89" s="1"/>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" s="1"/>
-      <c r="B90" s="10">
+      <c r="B90" s="9">
         <v>46143</v>
       </c>
       <c r="D90" s="1"/>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="1"/>
-      <c r="B91" s="10">
+      <c r="B91" s="9">
         <v>46144</v>
       </c>
       <c r="D91" s="1"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="1"/>
-      <c r="B92" s="10">
+      <c r="B92" s="9">
         <v>46145</v>
       </c>
       <c r="D92" s="1"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
-      <c r="B93" s="10">
+      <c r="B93" s="9">
         <v>46146</v>
       </c>
       <c r="D93" s="1"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="1"/>
-      <c r="B94" s="10">
+      <c r="B94" s="9">
         <v>46147</v>
       </c>
       <c r="D94" s="1"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="1"/>
-      <c r="B95" s="10">
+      <c r="B95" s="9">
         <v>46148</v>
       </c>
       <c r="D95" s="1"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="1"/>
-      <c r="B96" s="10">
+      <c r="B96" s="9">
         <v>46149</v>
       </c>
       <c r="D96" s="1"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="1"/>
-      <c r="B97" s="10">
+      <c r="B97" s="9">
         <v>46150</v>
       </c>
       <c r="D97" s="1"/>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" s="1"/>
-      <c r="B98" s="10">
+      <c r="B98" s="9">
         <v>46151</v>
       </c>
       <c r="D98" s="1"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" s="1"/>
-      <c r="B99" s="10">
+      <c r="B99" s="9">
         <v>46152</v>
       </c>
       <c r="D99" s="1"/>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" s="1"/>
-      <c r="B100" s="10">
+      <c r="B100" s="9">
         <v>46153</v>
       </c>
       <c r="D100" s="1"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="1"/>
-      <c r="B101" s="10">
+      <c r="B101" s="9">
         <v>46154</v>
       </c>
       <c r="D101" s="1"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="1"/>
-      <c r="B102" s="10">
+      <c r="B102" s="9">
         <v>46155</v>
       </c>
       <c r="D102" s="1"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" s="1"/>
-      <c r="B103" s="10">
+      <c r="B103" s="9">
         <v>46156</v>
       </c>
       <c r="D103" s="1"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" s="1"/>
-      <c r="B104" s="10">
+      <c r="B104" s="9">
         <v>46157</v>
       </c>
       <c r="D104" s="1"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" s="1"/>
-      <c r="B105" s="10">
+      <c r="B105" s="9">
         <v>46158</v>
       </c>
       <c r="D105" s="1"/>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" s="1"/>
-      <c r="B106" s="10">
+      <c r="B106" s="9">
         <v>46159</v>
       </c>
       <c r="D106" s="1"/>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" s="1"/>
-      <c r="B107" s="10">
+      <c r="B107" s="9">
         <v>46160</v>
       </c>
       <c r="D107" s="1"/>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" s="1"/>
-      <c r="B108" s="10">
+      <c r="B108" s="9">
         <v>46161</v>
       </c>
       <c r="D108" s="1"/>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" s="1"/>
-      <c r="B109" s="10">
+      <c r="B109" s="9">
         <v>46162</v>
       </c>
       <c r="D109" s="1"/>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" s="1"/>
-      <c r="B110" s="10">
+      <c r="B110" s="9">
         <v>46163</v>
       </c>
       <c r="D110" s="1"/>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" s="1"/>
-      <c r="B111" s="10">
+      <c r="B111" s="9">
         <v>46164</v>
       </c>
       <c r="D111" s="1"/>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" s="1"/>
-      <c r="B112" s="10">
+      <c r="B112" s="9">
         <v>46165</v>
       </c>
       <c r="D112" s="1"/>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" s="1"/>
-      <c r="B113" s="10">
+      <c r="B113" s="9">
         <v>46166</v>
       </c>
       <c r="D113" s="1"/>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" s="1"/>
-      <c r="B114" s="10">
+      <c r="B114" s="9">
         <v>46167</v>
       </c>
       <c r="D114" s="1"/>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" s="1"/>
-      <c r="B115" s="10">
+      <c r="B115" s="9">
         <v>46168</v>
       </c>
       <c r="D115" s="1"/>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" s="1"/>
-      <c r="B116" s="10">
+      <c r="B116" s="9">
         <v>46169</v>
       </c>
       <c r="D116" s="1"/>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" s="1"/>
-      <c r="B117" s="10">
+      <c r="B117" s="9">
         <v>46170</v>
       </c>
       <c r="D117" s="1"/>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" s="1"/>
-      <c r="B118" s="10">
+      <c r="B118" s="9">
         <v>46171</v>
       </c>
       <c r="D118" s="1"/>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" s="1"/>
-      <c r="B119" s="10">
+      <c r="B119" s="9">
         <v>46172</v>
       </c>
       <c r="D119" s="1"/>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" s="1"/>
-      <c r="B120" s="10">
+      <c r="B120" s="9">
         <v>46173</v>
       </c>
       <c r="D120" s="1"/>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" s="1"/>
-      <c r="B121" s="10">
+      <c r="B121" s="9">
         <v>46174</v>
       </c>
       <c r="D121" s="1"/>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" s="1"/>
-      <c r="B122" s="10">
+      <c r="B122" s="9">
         <v>46175</v>
       </c>
       <c r="D122" s="1"/>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" s="1"/>
-      <c r="B123" s="10">
+      <c r="B123" s="9">
         <v>46176</v>
       </c>
       <c r="D123" s="1"/>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" s="1"/>
-      <c r="B124" s="10">
+      <c r="B124" s="9">
         <v>46177</v>
       </c>
       <c r="D124" s="1"/>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" s="1"/>
-      <c r="B125" s="10">
+      <c r="B125" s="9">
         <v>46178</v>
       </c>
       <c r="D125" s="1"/>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" s="1"/>
-      <c r="B126" s="10">
+      <c r="B126" s="9">
         <v>46179</v>
       </c>
       <c r="D126" s="1"/>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" s="1"/>
-      <c r="B127" s="10">
+      <c r="B127" s="9">
         <v>46180</v>
       </c>
       <c r="D127" s="1"/>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" s="1"/>
-      <c r="B128" s="10">
+      <c r="B128" s="9">
         <v>46181</v>
       </c>
       <c r="D128" s="1"/>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" s="1"/>
-      <c r="B129" s="10">
+      <c r="B129" s="9">
         <v>46182</v>
       </c>
       <c r="D129" s="1"/>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" s="1"/>
-      <c r="B130" s="10">
+      <c r="B130" s="9">
         <v>46183</v>
       </c>
       <c r="D130" s="1"/>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" s="1"/>
-      <c r="B131" s="10">
+      <c r="B131" s="9">
         <v>46184</v>
       </c>
       <c r="D131" s="1"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" s="1"/>
-      <c r="B132" s="10">
+      <c r="B132" s="9">
         <v>46185</v>
       </c>
       <c r="D132" s="1"/>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" s="1"/>
-      <c r="B133" s="17">
+      <c r="B133" s="13">
         <v>46186</v>
       </c>
       <c r="D133" s="1"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" s="1"/>
-      <c r="B134" s="17">
+      <c r="B134" s="13">
         <v>46187</v>
       </c>
       <c r="D134" s="1"/>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" s="1"/>
-      <c r="B135" s="15">
+      <c r="B135" s="13">
         <v>46188</v>
       </c>
       <c r="D135" s="1"/>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" s="1"/>
-      <c r="B136" s="15">
+      <c r="B136" s="13">
         <v>46189</v>
       </c>
       <c r="D136" s="1"/>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" s="1"/>
-      <c r="B137" s="15">
+      <c r="B137" s="13">
         <v>46190</v>
       </c>
       <c r="D137" s="1"/>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" s="1"/>
-      <c r="B138" s="15">
+      <c r="B138" s="13">
         <v>46191</v>
       </c>
       <c r="D138" s="1"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" s="1"/>
-      <c r="B139" s="15">
+      <c r="B139" s="13">
         <v>46192</v>
       </c>
       <c r="D139" s="1"/>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" s="1"/>
-      <c r="B140" s="15">
+      <c r="B140" s="13">
         <v>46193</v>
       </c>
       <c r="D140" s="1"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" s="1"/>
-      <c r="B141" s="15">
+      <c r="B141" s="13">
         <v>46194</v>
       </c>
       <c r="D141" s="1"/>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" s="1"/>
-      <c r="B142" s="15">
+      <c r="B142" s="13">
         <v>46195</v>
       </c>
       <c r="D142" s="1"/>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" s="1"/>
-      <c r="B143" s="15">
+      <c r="B143" s="13">
         <v>46196</v>
       </c>
       <c r="D143" s="1"/>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" s="1"/>
-      <c r="B144" s="15">
+      <c r="B144" s="13">
         <v>46197</v>
       </c>
       <c r="D144" s="1"/>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" s="1"/>
-      <c r="B145" s="15">
+      <c r="B145" s="13">
         <v>46198</v>
       </c>
       <c r="D145" s="1"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" s="1"/>
-      <c r="B146" s="15">
+      <c r="B146" s="13">
         <v>46199</v>
       </c>
       <c r="D146" s="1"/>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" s="1"/>
-      <c r="B147" s="16">
+      <c r="B147" s="14">
         <v>46200</v>
       </c>
       <c r="D147" s="1"/>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" s="1"/>
-      <c r="B148" s="16">
+      <c r="B148" s="14">
         <v>46201</v>
       </c>
       <c r="D148" s="1"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" s="1"/>
-      <c r="B149" s="16">
+      <c r="B149" s="14">
         <v>46202</v>
       </c>
       <c r="D149" s="1"/>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B150" s="16">
+      <c r="B150" s="14">
         <v>46203</v>
       </c>
       <c r="D150" s="1"/>

</xml_diff>